<commit_message>
removed usless excel stuff
</commit_message>
<xml_diff>
--- a/calc_and_rack.xlsx
+++ b/calc_and_rack.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\l7aur\Desktop\CND\CNP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66AC6BDD-C523-43C3-8A25-2ACF385A89BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD9531D-7E98-4B24-81D9-CBBB9097B79B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A7CA0D7A-53D0-40E5-91E0-784DA3F57821}"/>
   </bookViews>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -116,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="170">
   <si>
     <t>Spatiu ocupat in U</t>
   </si>
@@ -338,9 +338,6 @@
   </si>
   <si>
     <t>From your design</t>
-  </si>
-  <si>
-    <t>should be between 30 and 60</t>
   </si>
   <si>
     <t>From detailed calcullus of prototype room/rooms</t>
@@ -1186,7 +1183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1239,6 +1236,26 @@
     <xf numFmtId="49" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="12" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1299,25 +1316,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1666,9 +1666,9 @@
     <col min="4" max="5" width="8.21875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" style="70" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" style="50" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.77734375" style="73" customWidth="1"/>
+    <col min="10" max="10" width="12.77734375" style="53" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1693,19 +1693,19 @@
       <c r="G1" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="H1" s="66" t="s">
+      <c r="H1" s="46" t="s">
         <v>53</v>
       </c>
       <c r="I1" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="71" t="s">
-        <v>158</v>
+      <c r="J1" s="51" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="40" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="40" t="s">
         <v>54</v>
@@ -1735,13 +1735,13 @@
         <f>2*F2*(G2+H2+6)</f>
         <v>352.79999999999995</v>
       </c>
-      <c r="J2" s="72" t="s">
-        <v>159</v>
+      <c r="J2" s="52" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="40" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3" s="40" t="s">
         <v>54</v>
@@ -1771,29 +1771,29 @@
         <f>2*F3*(G3+H3+6)</f>
         <v>325.32</v>
       </c>
-      <c r="J3" s="72" t="s">
-        <v>160</v>
+      <c r="J3" s="52" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="44" t="s">
-        <v>78</v>
-      </c>
-      <c r="B4" s="58" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="70" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="60"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="72"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="40" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B5" s="40" t="s">
         <v>54</v>
@@ -1823,13 +1823,13 @@
         <f>2*F5*(G5+H5+6)</f>
         <v>388.2</v>
       </c>
-      <c r="J5" s="72" t="s">
-        <v>161</v>
+      <c r="J5" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B6" s="40" t="s">
         <v>54</v>
@@ -1859,13 +1859,13 @@
         <f t="shared" ref="I6:I9" si="2">2*F6*(G6+H6+6)</f>
         <v>448.2</v>
       </c>
-      <c r="J6" s="72" t="s">
-        <v>161</v>
+      <c r="J6" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="40" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B7" s="40" t="s">
         <v>54</v>
@@ -1895,13 +1895,13 @@
         <f t="shared" si="2"/>
         <v>505.3</v>
       </c>
-      <c r="J7" s="72" t="s">
-        <v>161</v>
+      <c r="J7" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="40" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="40" t="s">
         <v>54</v>
@@ -1931,13 +1931,13 @@
         <f t="shared" si="2"/>
         <v>565.29999999999995</v>
       </c>
-      <c r="J8" s="72" t="s">
-        <v>161</v>
+      <c r="J8" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" s="40" t="s">
         <v>54</v>
@@ -1967,43 +1967,43 @@
         <f t="shared" si="2"/>
         <v>622.4</v>
       </c>
-      <c r="J9" s="72" t="s">
-        <v>161</v>
+      <c r="J9" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="43" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="46" t="s">
-        <v>155</v>
-      </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="48"/>
+        <v>83</v>
+      </c>
+      <c r="B10" s="58" t="s">
+        <v>154</v>
+      </c>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="59"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="59"/>
+      <c r="J10" s="60"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="43" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="49"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="51"/>
+        <v>84</v>
+      </c>
+      <c r="B11" s="61"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62"/>
+      <c r="J11" s="63"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="40" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B12" s="40" t="s">
         <v>54</v>
@@ -2033,13 +2033,13 @@
         <f>2*F12*(G12+H12+6)</f>
         <v>350</v>
       </c>
-      <c r="J12" s="72" t="s">
-        <v>162</v>
+      <c r="J12" s="52" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B13" s="40" t="s">
         <v>54</v>
@@ -2069,13 +2069,13 @@
         <f t="shared" ref="I13:I19" si="3">2*F13*(G13+H13+6)</f>
         <v>2178</v>
       </c>
-      <c r="J13" s="72" t="s">
-        <v>163</v>
+      <c r="J13" s="52" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B14" s="40" t="s">
         <v>54</v>
@@ -2105,13 +2105,13 @@
         <f t="shared" si="3"/>
         <v>1722.24</v>
       </c>
-      <c r="J14" s="72" t="s">
-        <v>164</v>
+      <c r="J14" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B15" s="40" t="s">
         <v>54</v>
@@ -2141,13 +2141,13 @@
         <f t="shared" si="3"/>
         <v>1836.48</v>
       </c>
-      <c r="J15" s="72" t="s">
-        <v>164</v>
+      <c r="J15" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B16" s="40" t="s">
         <v>54</v>
@@ -2177,13 +2177,13 @@
         <f t="shared" si="3"/>
         <v>1948.48</v>
       </c>
-      <c r="J16" s="72" t="s">
-        <v>164</v>
+      <c r="J16" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B17" s="40" t="s">
         <v>54</v>
@@ -2213,13 +2213,13 @@
         <f t="shared" si="3"/>
         <v>2062.7200000000003</v>
       </c>
-      <c r="J17" s="72" t="s">
-        <v>164</v>
+      <c r="J17" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="40" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B18" s="40" t="s">
         <v>54</v>
@@ -2249,13 +2249,13 @@
         <f t="shared" si="3"/>
         <v>2174.7200000000003</v>
       </c>
-      <c r="J18" s="72" t="s">
-        <v>164</v>
+      <c r="J18" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="40" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B19" s="40" t="s">
         <v>54</v>
@@ -2285,8 +2285,8 @@
         <f t="shared" si="3"/>
         <v>1500</v>
       </c>
-      <c r="J19" s="72" t="s">
-        <v>165</v>
+      <c r="J19" s="52" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -2302,7 +2302,7 @@
         <v>140</v>
       </c>
       <c r="G20" s="29"/>
-      <c r="H20" s="67"/>
+      <c r="H20" s="47"/>
       <c r="I20" s="29">
         <f>SUM(I2:I19)</f>
         <v>16980.16</v>
@@ -2316,12 +2316,12 @@
       <c r="E21" s="29"/>
       <c r="F21" s="29"/>
       <c r="G21" s="29"/>
-      <c r="H21" s="67"/>
+      <c r="H21" s="47"/>
       <c r="I21" s="29"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B22" s="40" t="s">
         <v>55</v>
@@ -2343,7 +2343,7 @@
       <c r="G22" s="39">
         <v>32</v>
       </c>
-      <c r="H22" s="68" cm="1">
+      <c r="H22" s="48" cm="1">
         <f t="array" ref="H22">_xlfn.CEILING.MATH(_xlfn.SWITCH(J22, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -2351,13 +2351,13 @@
         <f>2*F22*(G22+H22+6)</f>
         <v>880</v>
       </c>
-      <c r="J22" s="72" t="s">
-        <v>164</v>
+      <c r="J22" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="40" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B23" s="40" t="s">
         <v>55</v>
@@ -2379,7 +2379,7 @@
       <c r="G23" s="39">
         <v>27</v>
       </c>
-      <c r="H23" s="68" cm="1">
+      <c r="H23" s="48" cm="1">
         <f t="array" ref="H23">_xlfn.CEILING.MATH(_xlfn.SWITCH(J23, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -2387,43 +2387,43 @@
         <f>2*F23*(G23+H23+6)</f>
         <v>800</v>
       </c>
-      <c r="J23" s="72" t="s">
-        <v>164</v>
+      <c r="J23" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="43" t="s">
+        <v>153</v>
+      </c>
+      <c r="B24" s="58" t="s">
         <v>154</v>
       </c>
-      <c r="B24" s="46" t="s">
-        <v>155</v>
-      </c>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="47"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="47"/>
-      <c r="I24" s="47"/>
-      <c r="J24" s="48"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="59"/>
+      <c r="H24" s="59"/>
+      <c r="I24" s="59"/>
+      <c r="J24" s="60"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="43" t="s">
-        <v>151</v>
-      </c>
-      <c r="B25" s="49"/>
-      <c r="C25" s="50"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="51"/>
+        <v>150</v>
+      </c>
+      <c r="B25" s="61"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="62"/>
+      <c r="H25" s="62"/>
+      <c r="I25" s="62"/>
+      <c r="J25" s="63"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="40" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B26" s="40" t="s">
         <v>55</v>
@@ -2445,7 +2445,7 @@
       <c r="G26" s="39">
         <v>0.5</v>
       </c>
-      <c r="H26" s="68" cm="1">
+      <c r="H26" s="48" cm="1">
         <f t="array" ref="H26">_xlfn.CEILING.MATH(_xlfn.SWITCH(J26, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>14</v>
       </c>
@@ -2453,13 +2453,13 @@
         <f>2*F26*(G26+H26+6)</f>
         <v>820</v>
       </c>
-      <c r="J26" s="72" t="s">
-        <v>165</v>
+      <c r="J26" s="52" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="40" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B27" s="40" t="s">
         <v>55</v>
@@ -2481,7 +2481,7 @@
       <c r="G27" s="39">
         <v>45</v>
       </c>
-      <c r="H27" s="68" cm="1">
+      <c r="H27" s="48" cm="1">
         <f t="array" ref="H27">_xlfn.CEILING.MATH(_xlfn.SWITCH(J27, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>20</v>
       </c>
@@ -2489,13 +2489,13 @@
         <f t="shared" ref="I27:I30" si="6">2*F27*(G27+H27+6)</f>
         <v>1278</v>
       </c>
-      <c r="J27" s="72" t="s">
-        <v>166</v>
+      <c r="J27" s="52" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="40" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B28" s="40" t="s">
         <v>55</v>
@@ -2517,7 +2517,7 @@
       <c r="G28" s="39">
         <v>40</v>
       </c>
-      <c r="H28" s="68" cm="1">
+      <c r="H28" s="48" cm="1">
         <f t="array" ref="H28">_xlfn.CEILING.MATH(_xlfn.SWITCH(J28, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>20</v>
       </c>
@@ -2525,13 +2525,13 @@
         <f t="shared" si="6"/>
         <v>1188</v>
       </c>
-      <c r="J28" s="72" t="s">
-        <v>166</v>
+      <c r="J28" s="52" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="40" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" s="40" t="s">
         <v>55</v>
@@ -2553,7 +2553,7 @@
       <c r="G29" s="39">
         <v>12.54</v>
       </c>
-      <c r="H29" s="68" cm="1">
+      <c r="H29" s="48" cm="1">
         <f t="array" ref="H29">_xlfn.CEILING.MATH(_xlfn.SWITCH(J29, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -2561,13 +2561,13 @@
         <f t="shared" si="6"/>
         <v>438.48</v>
       </c>
-      <c r="J29" s="72" t="s">
-        <v>167</v>
+      <c r="J29" s="52" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="40" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B30" s="40" t="s">
         <v>55</v>
@@ -2589,7 +2589,7 @@
       <c r="G30" s="39">
         <v>21.88</v>
       </c>
-      <c r="H30" s="68" cm="1">
+      <c r="H30" s="48" cm="1">
         <f t="array" ref="H30">_xlfn.CEILING.MATH(_xlfn.SWITCH(J30, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -2597,29 +2597,29 @@
         <f t="shared" si="6"/>
         <v>550.55999999999995</v>
       </c>
-      <c r="J30" s="72" t="s">
-        <v>167</v>
+      <c r="J30" s="52" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="44" t="s">
-        <v>99</v>
-      </c>
-      <c r="B31" s="58" t="s">
+        <v>98</v>
+      </c>
+      <c r="B31" s="70" t="s">
         <v>55</v>
       </c>
-      <c r="C31" s="59"/>
-      <c r="D31" s="59"/>
-      <c r="E31" s="59"/>
-      <c r="F31" s="59"/>
-      <c r="G31" s="59"/>
-      <c r="H31" s="59"/>
-      <c r="I31" s="59"/>
-      <c r="J31" s="60"/>
+      <c r="C31" s="71"/>
+      <c r="D31" s="71"/>
+      <c r="E31" s="71"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="71"/>
+      <c r="H31" s="71"/>
+      <c r="I31" s="71"/>
+      <c r="J31" s="72"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B32" s="40" t="s">
         <v>55</v>
@@ -2649,13 +2649,13 @@
         <f>2*F32*(G32+H32+6)</f>
         <v>305</v>
       </c>
-      <c r="J32" s="72" t="s">
-        <v>168</v>
+      <c r="J32" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B33" s="40" t="s">
         <v>55</v>
@@ -2685,13 +2685,13 @@
         <f t="shared" ref="I33:I36" si="10">2*F33*(G33+H33+6)</f>
         <v>360</v>
       </c>
-      <c r="J33" s="72" t="s">
-        <v>168</v>
+      <c r="J33" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="40" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B34" s="40" t="s">
         <v>55</v>
@@ -2721,13 +2721,13 @@
         <f t="shared" si="10"/>
         <v>415</v>
       </c>
-      <c r="J34" s="72" t="s">
-        <v>168</v>
+      <c r="J34" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="40" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B35" s="40" t="s">
         <v>55</v>
@@ -2757,13 +2757,13 @@
         <f t="shared" si="10"/>
         <v>470</v>
       </c>
-      <c r="J35" s="72" t="s">
-        <v>168</v>
+      <c r="J35" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="40" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B36" s="40" t="s">
         <v>55</v>
@@ -2793,43 +2793,43 @@
         <f t="shared" si="10"/>
         <v>525</v>
       </c>
-      <c r="J36" s="72" t="s">
-        <v>168</v>
+      <c r="J36" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="43" t="s">
-        <v>156</v>
-      </c>
-      <c r="B37" s="52" t="s">
         <v>155</v>
       </c>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="53"/>
-      <c r="G37" s="53"/>
-      <c r="H37" s="53"/>
-      <c r="I37" s="53"/>
-      <c r="J37" s="54"/>
+      <c r="B37" s="64" t="s">
+        <v>154</v>
+      </c>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="66"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="43" t="s">
-        <v>157</v>
-      </c>
-      <c r="B38" s="55"/>
-      <c r="C38" s="56"/>
-      <c r="D38" s="56"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="56"/>
-      <c r="H38" s="56"/>
-      <c r="I38" s="56"/>
-      <c r="J38" s="57"/>
+        <v>156</v>
+      </c>
+      <c r="B38" s="67"/>
+      <c r="C38" s="68"/>
+      <c r="D38" s="68"/>
+      <c r="E38" s="68"/>
+      <c r="F38" s="68"/>
+      <c r="G38" s="68"/>
+      <c r="H38" s="68"/>
+      <c r="I38" s="68"/>
+      <c r="J38" s="69"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="40" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B39" s="40" t="s">
         <v>55</v>
@@ -2859,13 +2859,13 @@
         <f>2*F39*(G39+H39+6)</f>
         <v>552</v>
       </c>
-      <c r="J39" s="72" t="s">
-        <v>169</v>
+      <c r="J39" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B40" s="40" t="s">
         <v>55</v>
@@ -2895,13 +2895,13 @@
         <f t="shared" ref="I40:I44" si="11">2*F40*(G40+H40+6)</f>
         <v>581</v>
       </c>
-      <c r="J40" s="72" t="s">
-        <v>169</v>
+      <c r="J40" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="40" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B41" s="40" t="s">
         <v>55</v>
@@ -2931,13 +2931,13 @@
         <f t="shared" si="11"/>
         <v>665</v>
       </c>
-      <c r="J41" s="72" t="s">
-        <v>169</v>
+      <c r="J41" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B42" s="40" t="s">
         <v>55</v>
@@ -2967,13 +2967,13 @@
         <f t="shared" si="11"/>
         <v>749</v>
       </c>
-      <c r="J42" s="72" t="s">
-        <v>169</v>
+      <c r="J42" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B43" s="40" t="s">
         <v>55</v>
@@ -3003,13 +3003,13 @@
         <f t="shared" si="11"/>
         <v>833</v>
       </c>
-      <c r="J43" s="72" t="s">
-        <v>169</v>
+      <c r="J43" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="40" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B44" s="40" t="s">
         <v>55</v>
@@ -3039,8 +3039,8 @@
         <f t="shared" si="11"/>
         <v>917</v>
       </c>
-      <c r="J44" s="72" t="s">
-        <v>169</v>
+      <c r="J44" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
@@ -3056,7 +3056,7 @@
         <v>134</v>
       </c>
       <c r="G45" s="29"/>
-      <c r="H45" s="67"/>
+      <c r="H45" s="47"/>
       <c r="I45" s="29">
         <f>SUM(I22:I44)</f>
         <v>12327.039999999999</v>
@@ -3070,12 +3070,12 @@
       <c r="E46" s="29"/>
       <c r="F46" s="29"/>
       <c r="G46" s="29"/>
-      <c r="H46" s="67"/>
+      <c r="H46" s="47"/>
       <c r="I46" s="29"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="40" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B47" s="39" t="s">
         <v>56</v>
@@ -3097,7 +3097,7 @@
       <c r="G47" s="39">
         <v>9.4</v>
       </c>
-      <c r="H47" s="68" cm="1">
+      <c r="H47" s="48" cm="1">
         <f t="array" ref="H47">_xlfn.CEILING.MATH(_xlfn.SWITCH(J47, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>14</v>
       </c>
@@ -3105,13 +3105,13 @@
         <f>2*F47*(G47+H47+6)</f>
         <v>352.79999999999995</v>
       </c>
-      <c r="J47" s="72" t="s">
-        <v>159</v>
+      <c r="J47" s="52" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="40" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B48" s="39" t="s">
         <v>56</v>
@@ -3133,7 +3133,7 @@
       <c r="G48" s="39">
         <v>16.11</v>
       </c>
-      <c r="H48" s="68" cm="1">
+      <c r="H48" s="48" cm="1">
         <f t="array" ref="H48">_xlfn.CEILING.MATH(_xlfn.SWITCH(J48, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>5</v>
       </c>
@@ -3141,29 +3141,29 @@
         <f>2*F48*(G48+H48+6)</f>
         <v>325.32</v>
       </c>
-      <c r="J48" s="72" t="s">
-        <v>160</v>
+      <c r="J48" s="52" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="44" t="s">
-        <v>113</v>
-      </c>
-      <c r="B49" s="61" t="s">
+        <v>112</v>
+      </c>
+      <c r="B49" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="63"/>
+      <c r="C49" s="74"/>
+      <c r="D49" s="74"/>
+      <c r="E49" s="74"/>
+      <c r="F49" s="74"/>
+      <c r="G49" s="74"/>
+      <c r="H49" s="74"/>
+      <c r="I49" s="74"/>
+      <c r="J49" s="75"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="40" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B50" s="39" t="s">
         <v>56</v>
@@ -3185,7 +3185,7 @@
       <c r="G50" s="39">
         <v>21.82</v>
       </c>
-      <c r="H50" s="68" cm="1">
+      <c r="H50" s="48" cm="1">
         <f t="array" ref="H50">_xlfn.CEILING.MATH(_xlfn.SWITCH(J50, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>11</v>
       </c>
@@ -3193,13 +3193,13 @@
         <f>2*F50*(G50+H50+6)</f>
         <v>388.2</v>
       </c>
-      <c r="J50" s="72" t="s">
-        <v>161</v>
+      <c r="J50" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="40" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B51" s="39" t="s">
         <v>56</v>
@@ -3221,7 +3221,7 @@
       <c r="G51" s="39">
         <v>27.82</v>
       </c>
-      <c r="H51" s="68" cm="1">
+      <c r="H51" s="48" cm="1">
         <f t="array" ref="H51">_xlfn.CEILING.MATH(_xlfn.SWITCH(J51, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>11</v>
       </c>
@@ -3229,13 +3229,13 @@
         <f t="shared" ref="I51:I54" si="15">2*F51*(G51+H51+6)</f>
         <v>448.2</v>
       </c>
-      <c r="J51" s="72" t="s">
-        <v>161</v>
+      <c r="J51" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="40" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B52" s="39" t="s">
         <v>56</v>
@@ -3257,7 +3257,7 @@
       <c r="G52" s="39">
         <v>33.53</v>
       </c>
-      <c r="H52" s="68" cm="1">
+      <c r="H52" s="48" cm="1">
         <f t="array" ref="H52">_xlfn.CEILING.MATH(_xlfn.SWITCH(J52, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>11</v>
       </c>
@@ -3265,13 +3265,13 @@
         <f t="shared" si="15"/>
         <v>505.3</v>
       </c>
-      <c r="J52" s="72" t="s">
-        <v>161</v>
+      <c r="J52" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="40" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B53" s="39" t="s">
         <v>56</v>
@@ -3293,7 +3293,7 @@
       <c r="G53" s="39">
         <v>39.53</v>
       </c>
-      <c r="H53" s="68" cm="1">
+      <c r="H53" s="48" cm="1">
         <f t="array" ref="H53">_xlfn.CEILING.MATH(_xlfn.SWITCH(J53, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>11</v>
       </c>
@@ -3301,13 +3301,13 @@
         <f t="shared" si="15"/>
         <v>565.29999999999995</v>
       </c>
-      <c r="J53" s="72" t="s">
-        <v>161</v>
+      <c r="J53" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="40" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B54" s="39" t="s">
         <v>56</v>
@@ -3329,7 +3329,7 @@
       <c r="G54" s="39">
         <v>45.24</v>
       </c>
-      <c r="H54" s="68" cm="1">
+      <c r="H54" s="48" cm="1">
         <f t="array" ref="H54">_xlfn.CEILING.MATH(_xlfn.SWITCH(J54, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>11</v>
       </c>
@@ -3337,43 +3337,43 @@
         <f t="shared" si="15"/>
         <v>622.4</v>
       </c>
-      <c r="J54" s="72" t="s">
-        <v>161</v>
+      <c r="J54" s="52" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="B55" s="46" t="s">
-        <v>155</v>
-      </c>
-      <c r="C55" s="47"/>
-      <c r="D55" s="47"/>
-      <c r="E55" s="47"/>
-      <c r="F55" s="47"/>
-      <c r="G55" s="47"/>
-      <c r="H55" s="47"/>
-      <c r="I55" s="47"/>
-      <c r="J55" s="48"/>
+        <v>118</v>
+      </c>
+      <c r="B55" s="58" t="s">
+        <v>154</v>
+      </c>
+      <c r="C55" s="59"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="59"/>
+      <c r="F55" s="59"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="59"/>
+      <c r="I55" s="59"/>
+      <c r="J55" s="60"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="43" t="s">
-        <v>120</v>
-      </c>
-      <c r="B56" s="49"/>
-      <c r="C56" s="50"/>
-      <c r="D56" s="50"/>
-      <c r="E56" s="50"/>
-      <c r="F56" s="50"/>
-      <c r="G56" s="50"/>
-      <c r="H56" s="50"/>
-      <c r="I56" s="50"/>
-      <c r="J56" s="51"/>
+        <v>119</v>
+      </c>
+      <c r="B56" s="61"/>
+      <c r="C56" s="62"/>
+      <c r="D56" s="62"/>
+      <c r="E56" s="62"/>
+      <c r="F56" s="62"/>
+      <c r="G56" s="62"/>
+      <c r="H56" s="62"/>
+      <c r="I56" s="62"/>
+      <c r="J56" s="63"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="40" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B57" s="39" t="s">
         <v>56</v>
@@ -3395,7 +3395,7 @@
       <c r="G57" s="39">
         <v>0.5</v>
       </c>
-      <c r="H57" s="68" cm="1">
+      <c r="H57" s="48" cm="1">
         <f t="array" ref="H57">_xlfn.CEILING.MATH(_xlfn.SWITCH(J57, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>11</v>
       </c>
@@ -3403,13 +3403,13 @@
         <f>2*F57*(G57+H57+6)</f>
         <v>350</v>
       </c>
-      <c r="J57" s="72" t="s">
-        <v>162</v>
+      <c r="J57" s="52" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B58" s="39" t="s">
         <v>56</v>
@@ -3431,7 +3431,7 @@
       <c r="G58" s="39">
         <v>5</v>
       </c>
-      <c r="H58" s="68" cm="1">
+      <c r="H58" s="48" cm="1">
         <f t="array" ref="H58">_xlfn.CEILING.MATH(_xlfn.SWITCH(J58, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>22</v>
       </c>
@@ -3439,13 +3439,13 @@
         <f t="shared" ref="I58:I64" si="16">2*F58*(G58+H58+6)</f>
         <v>2178</v>
       </c>
-      <c r="J58" s="72" t="s">
-        <v>163</v>
+      <c r="J58" s="52" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B59" s="39" t="s">
         <v>56</v>
@@ -3467,7 +3467,7 @@
       <c r="G59" s="39">
         <v>84.64</v>
       </c>
-      <c r="H59" s="68" cm="1">
+      <c r="H59" s="48" cm="1">
         <f t="array" ref="H59">_xlfn.CEILING.MATH(_xlfn.SWITCH(J59, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3475,13 +3475,13 @@
         <f t="shared" si="16"/>
         <v>1722.24</v>
       </c>
-      <c r="J59" s="72" t="s">
-        <v>164</v>
+      <c r="J59" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="40" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B60" s="39" t="s">
         <v>56</v>
@@ -3503,7 +3503,7 @@
       <c r="G60" s="39">
         <v>91.78</v>
       </c>
-      <c r="H60" s="68" cm="1">
+      <c r="H60" s="48" cm="1">
         <f t="array" ref="H60">_xlfn.CEILING.MATH(_xlfn.SWITCH(J60, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3511,13 +3511,13 @@
         <f t="shared" si="16"/>
         <v>1836.48</v>
       </c>
-      <c r="J60" s="72" t="s">
-        <v>164</v>
+      <c r="J60" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="40" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B61" s="39" t="s">
         <v>56</v>
@@ -3539,7 +3539,7 @@
       <c r="G61" s="39">
         <v>98.78</v>
       </c>
-      <c r="H61" s="68" cm="1">
+      <c r="H61" s="48" cm="1">
         <f t="array" ref="H61">_xlfn.CEILING.MATH(_xlfn.SWITCH(J61, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3547,13 +3547,13 @@
         <f t="shared" si="16"/>
         <v>1948.48</v>
       </c>
-      <c r="J61" s="72" t="s">
-        <v>164</v>
+      <c r="J61" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="40" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B62" s="39" t="s">
         <v>56</v>
@@ -3575,7 +3575,7 @@
       <c r="G62" s="39">
         <v>105.92</v>
       </c>
-      <c r="H62" s="68" cm="1">
+      <c r="H62" s="48" cm="1">
         <f t="array" ref="H62">_xlfn.CEILING.MATH(_xlfn.SWITCH(J62, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3583,13 +3583,13 @@
         <f t="shared" si="16"/>
         <v>2062.7200000000003</v>
       </c>
-      <c r="J62" s="72" t="s">
-        <v>164</v>
+      <c r="J62" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="40" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B63" s="39" t="s">
         <v>56</v>
@@ -3611,7 +3611,7 @@
       <c r="G63" s="39">
         <v>112.92</v>
       </c>
-      <c r="H63" s="68" cm="1">
+      <c r="H63" s="48" cm="1">
         <f t="array" ref="H63">_xlfn.CEILING.MATH(_xlfn.SWITCH(J63, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3619,13 +3619,13 @@
         <f t="shared" si="16"/>
         <v>2174.7200000000003</v>
       </c>
-      <c r="J63" s="72" t="s">
-        <v>164</v>
+      <c r="J63" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="40" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B64" s="39" t="s">
         <v>56</v>
@@ -3647,7 +3647,7 @@
       <c r="G64" s="39">
         <v>17.5</v>
       </c>
-      <c r="H64" s="68" cm="1">
+      <c r="H64" s="48" cm="1">
         <f t="array" ref="H64">_xlfn.CEILING.MATH(_xlfn.SWITCH(J64, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>14</v>
       </c>
@@ -3655,8 +3655,8 @@
         <f t="shared" si="16"/>
         <v>1500</v>
       </c>
-      <c r="J64" s="72" t="s">
-        <v>165</v>
+      <c r="J64" s="52" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
@@ -3672,7 +3672,7 @@
         <v>140</v>
       </c>
       <c r="G65" s="29"/>
-      <c r="H65" s="67"/>
+      <c r="H65" s="47"/>
       <c r="I65" s="29">
         <f>SUM(I47:I64)</f>
         <v>16980.16</v>
@@ -3686,12 +3686,12 @@
       <c r="E66" s="29"/>
       <c r="F66" s="29"/>
       <c r="G66" s="29"/>
-      <c r="H66" s="67"/>
+      <c r="H66" s="47"/>
       <c r="I66" s="29"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="40" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B67" s="40" t="s">
         <v>57</v>
@@ -3713,7 +3713,7 @@
       <c r="G67" s="39">
         <v>32</v>
       </c>
-      <c r="H67" s="68" cm="1">
+      <c r="H67" s="48" cm="1">
         <f t="array" ref="H67">_xlfn.CEILING.MATH(_xlfn.SWITCH(J67, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3721,13 +3721,13 @@
         <f>2*F67*(G67+H67+6)</f>
         <v>880</v>
       </c>
-      <c r="J67" s="72" t="s">
-        <v>164</v>
+      <c r="J67" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="40" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B68" s="40" t="s">
         <v>57</v>
@@ -3749,7 +3749,7 @@
       <c r="G68" s="39">
         <v>27</v>
       </c>
-      <c r="H68" s="68" cm="1">
+      <c r="H68" s="48" cm="1">
         <f t="array" ref="H68">_xlfn.CEILING.MATH(_xlfn.SWITCH(J68, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3757,43 +3757,43 @@
         <f>2*F68*(G68+H68+6)</f>
         <v>800</v>
       </c>
-      <c r="J68" s="72" t="s">
-        <v>164</v>
+      <c r="J68" s="52" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="43" t="s">
-        <v>150</v>
-      </c>
-      <c r="B69" s="46" t="s">
-        <v>155</v>
-      </c>
-      <c r="C69" s="47"/>
-      <c r="D69" s="47"/>
-      <c r="E69" s="47"/>
-      <c r="F69" s="47"/>
-      <c r="G69" s="47"/>
-      <c r="H69" s="47"/>
-      <c r="I69" s="47"/>
-      <c r="J69" s="48"/>
+        <v>149</v>
+      </c>
+      <c r="B69" s="58" t="s">
+        <v>154</v>
+      </c>
+      <c r="C69" s="59"/>
+      <c r="D69" s="59"/>
+      <c r="E69" s="59"/>
+      <c r="F69" s="59"/>
+      <c r="G69" s="59"/>
+      <c r="H69" s="59"/>
+      <c r="I69" s="59"/>
+      <c r="J69" s="60"/>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="43" t="s">
-        <v>147</v>
-      </c>
-      <c r="B70" s="49"/>
-      <c r="C70" s="50"/>
-      <c r="D70" s="50"/>
-      <c r="E70" s="50"/>
-      <c r="F70" s="50"/>
-      <c r="G70" s="50"/>
-      <c r="H70" s="50"/>
-      <c r="I70" s="50"/>
-      <c r="J70" s="51"/>
+        <v>146</v>
+      </c>
+      <c r="B70" s="61"/>
+      <c r="C70" s="62"/>
+      <c r="D70" s="62"/>
+      <c r="E70" s="62"/>
+      <c r="F70" s="62"/>
+      <c r="G70" s="62"/>
+      <c r="H70" s="62"/>
+      <c r="I70" s="62"/>
+      <c r="J70" s="63"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B71" s="40" t="s">
         <v>57</v>
@@ -3815,7 +3815,7 @@
       <c r="G71" s="39">
         <v>0.5</v>
       </c>
-      <c r="H71" s="68" cm="1">
+      <c r="H71" s="48" cm="1">
         <f t="array" ref="H71">_xlfn.CEILING.MATH(_xlfn.SWITCH(J71, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>14</v>
       </c>
@@ -3823,13 +3823,13 @@
         <f>2*F71*(G71+H71+6)</f>
         <v>820</v>
       </c>
-      <c r="J71" s="72" t="s">
-        <v>165</v>
+      <c r="J71" s="52" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="40" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B72" s="40" t="s">
         <v>57</v>
@@ -3851,7 +3851,7 @@
       <c r="G72" s="39">
         <v>56.07</v>
       </c>
-      <c r="H72" s="68" cm="1">
+      <c r="H72" s="48" cm="1">
         <f t="array" ref="H72">_xlfn.CEILING.MATH(_xlfn.SWITCH(J72, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>17</v>
       </c>
@@ -3859,13 +3859,13 @@
         <f t="shared" ref="I72:I74" si="21">2*F72*(G72+H72+6)</f>
         <v>1106.98</v>
       </c>
-      <c r="J72" s="72" t="s">
-        <v>170</v>
+      <c r="J72" s="52" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="40" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B73" s="40" t="s">
         <v>57</v>
@@ -3887,7 +3887,7 @@
       <c r="G73" s="39">
         <v>12.54</v>
       </c>
-      <c r="H73" s="68" cm="1">
+      <c r="H73" s="48" cm="1">
         <f t="array" ref="H73">_xlfn.CEILING.MATH(_xlfn.SWITCH(J73, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -3895,13 +3895,13 @@
         <f t="shared" si="21"/>
         <v>438.48</v>
       </c>
-      <c r="J73" s="72" t="s">
-        <v>167</v>
+      <c r="J73" s="52" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="40" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B74" s="40" t="s">
         <v>57</v>
@@ -3923,7 +3923,7 @@
       <c r="G74" s="39">
         <v>21.88</v>
       </c>
-      <c r="H74" s="68" cm="1">
+      <c r="H74" s="48" cm="1">
         <f t="array" ref="H74">_xlfn.CEILING.MATH(_xlfn.SWITCH(J74, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -3931,29 +3931,29 @@
         <f t="shared" si="21"/>
         <v>550.55999999999995</v>
       </c>
-      <c r="J74" s="72" t="s">
-        <v>167</v>
+      <c r="J74" s="52" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="44" t="s">
-        <v>133</v>
-      </c>
-      <c r="B75" s="58" t="s">
+        <v>132</v>
+      </c>
+      <c r="B75" s="70" t="s">
         <v>57</v>
       </c>
-      <c r="C75" s="59"/>
-      <c r="D75" s="59"/>
-      <c r="E75" s="59"/>
-      <c r="F75" s="59"/>
-      <c r="G75" s="59"/>
-      <c r="H75" s="59"/>
-      <c r="I75" s="59"/>
-      <c r="J75" s="60"/>
+      <c r="C75" s="71"/>
+      <c r="D75" s="71"/>
+      <c r="E75" s="71"/>
+      <c r="F75" s="71"/>
+      <c r="G75" s="71"/>
+      <c r="H75" s="71"/>
+      <c r="I75" s="71"/>
+      <c r="J75" s="72"/>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="40" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B76" s="40" t="s">
         <v>57</v>
@@ -3975,7 +3975,7 @@
       <c r="G76" s="39">
         <v>11.5</v>
       </c>
-      <c r="H76" s="68" cm="1">
+      <c r="H76" s="48" cm="1">
         <f t="array" ref="H76">_xlfn.CEILING.MATH(_xlfn.SWITCH(J76, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>13</v>
       </c>
@@ -3983,13 +3983,13 @@
         <f>2*F76*(G76+H76+6)</f>
         <v>122</v>
       </c>
-      <c r="J76" s="72" t="s">
-        <v>168</v>
+      <c r="J76" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="40" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B77" s="40" t="s">
         <v>57</v>
@@ -4011,7 +4011,7 @@
       <c r="G77" s="39">
         <v>17</v>
       </c>
-      <c r="H77" s="68" cm="1">
+      <c r="H77" s="48" cm="1">
         <f t="array" ref="H77">_xlfn.CEILING.MATH(_xlfn.SWITCH(J77, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>13</v>
       </c>
@@ -4019,13 +4019,13 @@
         <f t="shared" ref="I77:I80" si="23">2*F77*(G77+H77+6)</f>
         <v>360</v>
       </c>
-      <c r="J77" s="72" t="s">
-        <v>168</v>
+      <c r="J77" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="40" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B78" s="40" t="s">
         <v>57</v>
@@ -4047,7 +4047,7 @@
       <c r="G78" s="39">
         <v>22.5</v>
       </c>
-      <c r="H78" s="68" cm="1">
+      <c r="H78" s="48" cm="1">
         <f t="array" ref="H78">_xlfn.CEILING.MATH(_xlfn.SWITCH(J78, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>13</v>
       </c>
@@ -4055,13 +4055,13 @@
         <f t="shared" si="23"/>
         <v>415</v>
       </c>
-      <c r="J78" s="72" t="s">
-        <v>168</v>
+      <c r="J78" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="40" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B79" s="40" t="s">
         <v>57</v>
@@ -4083,7 +4083,7 @@
       <c r="G79" s="39">
         <v>28</v>
       </c>
-      <c r="H79" s="68" cm="1">
+      <c r="H79" s="48" cm="1">
         <f t="array" ref="H79">_xlfn.CEILING.MATH(_xlfn.SWITCH(J79, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>13</v>
       </c>
@@ -4091,13 +4091,13 @@
         <f t="shared" si="23"/>
         <v>470</v>
       </c>
-      <c r="J79" s="72" t="s">
-        <v>168</v>
+      <c r="J79" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B80" s="40" t="s">
         <v>57</v>
@@ -4119,7 +4119,7 @@
       <c r="G80" s="39">
         <v>33.5</v>
       </c>
-      <c r="H80" s="68" cm="1">
+      <c r="H80" s="48" cm="1">
         <f t="array" ref="H80">_xlfn.CEILING.MATH(_xlfn.SWITCH(J80, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>13</v>
       </c>
@@ -4127,43 +4127,43 @@
         <f t="shared" si="23"/>
         <v>525</v>
       </c>
-      <c r="J80" s="72" t="s">
-        <v>168</v>
+      <c r="J80" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="43" t="s">
-        <v>139</v>
-      </c>
-      <c r="B81" s="52" t="s">
-        <v>155</v>
-      </c>
-      <c r="C81" s="53"/>
-      <c r="D81" s="53"/>
-      <c r="E81" s="53"/>
-      <c r="F81" s="53"/>
-      <c r="G81" s="53"/>
-      <c r="H81" s="53"/>
-      <c r="I81" s="53"/>
-      <c r="J81" s="54"/>
+        <v>138</v>
+      </c>
+      <c r="B81" s="64" t="s">
+        <v>154</v>
+      </c>
+      <c r="C81" s="65"/>
+      <c r="D81" s="65"/>
+      <c r="E81" s="65"/>
+      <c r="F81" s="65"/>
+      <c r="G81" s="65"/>
+      <c r="H81" s="65"/>
+      <c r="I81" s="65"/>
+      <c r="J81" s="66"/>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="43" t="s">
-        <v>140</v>
-      </c>
-      <c r="B82" s="55"/>
-      <c r="C82" s="56"/>
-      <c r="D82" s="56"/>
-      <c r="E82" s="56"/>
-      <c r="F82" s="56"/>
-      <c r="G82" s="56"/>
-      <c r="H82" s="56"/>
-      <c r="I82" s="56"/>
-      <c r="J82" s="57"/>
+        <v>139</v>
+      </c>
+      <c r="B82" s="67"/>
+      <c r="C82" s="68"/>
+      <c r="D82" s="68"/>
+      <c r="E82" s="68"/>
+      <c r="F82" s="68"/>
+      <c r="G82" s="68"/>
+      <c r="H82" s="68"/>
+      <c r="I82" s="68"/>
+      <c r="J82" s="69"/>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="40" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B83" s="40" t="s">
         <v>57</v>
@@ -4185,7 +4185,7 @@
       <c r="G83" s="39">
         <v>10.5</v>
       </c>
-      <c r="H83" s="68" cm="1">
+      <c r="H83" s="48" cm="1">
         <f t="array" ref="H83">_xlfn.CEILING.MATH(_xlfn.SWITCH(J83, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -4193,13 +4193,13 @@
         <f>2*F83*(G83+H83+6)</f>
         <v>621</v>
       </c>
-      <c r="J83" s="72" t="s">
-        <v>169</v>
+      <c r="J83" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="40" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B84" s="40" t="s">
         <v>57</v>
@@ -4221,7 +4221,7 @@
       <c r="G84" s="39">
         <v>17.5</v>
       </c>
-      <c r="H84" s="68" cm="1">
+      <c r="H84" s="48" cm="1">
         <f t="array" ref="H84">_xlfn.CEILING.MATH(_xlfn.SWITCH(J84, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -4229,13 +4229,13 @@
         <f t="shared" ref="I84:I88" si="25">2*F84*(G84+H84+6)</f>
         <v>747</v>
       </c>
-      <c r="J84" s="72" t="s">
-        <v>169</v>
+      <c r="J84" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="40" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B85" s="40" t="s">
         <v>57</v>
@@ -4257,7 +4257,7 @@
       <c r="G85" s="39">
         <v>23.5</v>
       </c>
-      <c r="H85" s="68" cm="1">
+      <c r="H85" s="48" cm="1">
         <f t="array" ref="H85">_xlfn.CEILING.MATH(_xlfn.SWITCH(J85, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -4265,13 +4265,13 @@
         <f t="shared" si="25"/>
         <v>665</v>
       </c>
-      <c r="J85" s="72" t="s">
-        <v>169</v>
+      <c r="J85" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="40" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B86" s="40" t="s">
         <v>57</v>
@@ -4293,7 +4293,7 @@
       <c r="G86" s="39">
         <v>29.5</v>
       </c>
-      <c r="H86" s="68" cm="1">
+      <c r="H86" s="48" cm="1">
         <f t="array" ref="H86">_xlfn.CEILING.MATH(_xlfn.SWITCH(J86, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -4301,13 +4301,13 @@
         <f t="shared" si="25"/>
         <v>749</v>
       </c>
-      <c r="J86" s="72" t="s">
-        <v>169</v>
+      <c r="J86" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="40" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B87" s="40" t="s">
         <v>57</v>
@@ -4329,7 +4329,7 @@
       <c r="G87" s="39">
         <v>35.5</v>
       </c>
-      <c r="H87" s="68" cm="1">
+      <c r="H87" s="48" cm="1">
         <f t="array" ref="H87">_xlfn.CEILING.MATH(_xlfn.SWITCH(J87, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -4337,13 +4337,13 @@
         <f t="shared" si="25"/>
         <v>833</v>
       </c>
-      <c r="J87" s="72" t="s">
-        <v>169</v>
+      <c r="J87" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B88" s="40" t="s">
         <v>57</v>
@@ -4365,7 +4365,7 @@
       <c r="G88" s="39">
         <v>41.5</v>
       </c>
-      <c r="H88" s="68" cm="1">
+      <c r="H88" s="48" cm="1">
         <f t="array" ref="H88">_xlfn.CEILING.MATH(_xlfn.SWITCH(J88, "A", 13.21, "B", 4.86, "C", 10.56, "D", 10.87, "E", 16.75, "F", 22, "G", 13.2, "H", 19.3, "I", 17.5, "J", 12.8, "K", 17.3, "L", 17, -1))</f>
         <v>18</v>
       </c>
@@ -4373,8 +4373,8 @@
         <f t="shared" si="25"/>
         <v>917</v>
       </c>
-      <c r="J88" s="72" t="s">
-        <v>169</v>
+      <c r="J88" s="52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.3">
@@ -4390,7 +4390,7 @@
         <v>123</v>
       </c>
       <c r="G89" s="29"/>
-      <c r="H89" s="67"/>
+      <c r="H89" s="47"/>
       <c r="I89" s="29">
         <f>SUM(I67:I88)</f>
         <v>11020.02</v>
@@ -4409,14 +4409,14 @@
         <v>537</v>
       </c>
       <c r="G91" s="37"/>
-      <c r="H91" s="69"/>
+      <c r="H91" s="49"/>
       <c r="I91" s="37">
         <f>I89+I65+I45+I20</f>
         <v>57307.380000000005</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H93" s="67" t="s">
+      <c r="H93" s="47" t="s">
         <v>68</v>
       </c>
       <c r="I93" s="29">
@@ -4425,7 +4425,7 @@
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H94" s="67" t="s">
+      <c r="H94" s="47" t="s">
         <v>69</v>
       </c>
       <c r="I94" s="29">
@@ -4434,52 +4434,57 @@
       </c>
     </row>
     <row r="96" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+      <c r="A96" s="78" t="s">
         <v>70</v>
       </c>
+      <c r="B96" s="78"/>
       <c r="C96" s="37">
         <f>I91/(F91*2)</f>
         <v>53.358826815642459</v>
       </c>
-      <c r="E96" t="s">
+    </row>
+    <row r="98" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A98" s="54" t="s">
+        <v>71</v>
+      </c>
+      <c r="B98" s="54"/>
+      <c r="C98" s="54"/>
+      <c r="D98" s="54"/>
+      <c r="E98" s="54"/>
+      <c r="F98" s="54"/>
+      <c r="G98" s="54"/>
+      <c r="H98" s="54"/>
+    </row>
+    <row r="99" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A99" s="55" t="s">
+        <v>72</v>
+      </c>
+      <c r="B99" s="55"/>
+    </row>
+    <row r="100" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A100" s="56" t="s">
+        <v>73</v>
+      </c>
+      <c r="B100" s="56"/>
+    </row>
+    <row r="101" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A101" s="57" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="98" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A98" s="74" t="s">
-        <v>71</v>
-      </c>
-      <c r="B98" s="74"/>
-      <c r="C98" s="74"/>
-      <c r="D98" s="74"/>
-      <c r="E98" s="74"/>
-      <c r="F98" s="74"/>
-      <c r="G98" s="74"/>
-      <c r="H98" s="74"/>
-    </row>
-    <row r="99" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A99" s="75" t="s">
-        <v>72</v>
-      </c>
-      <c r="B99" s="75"/>
-    </row>
-    <row r="100" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A100" s="76" t="s">
-        <v>73</v>
-      </c>
-      <c r="B100" s="76"/>
-    </row>
-    <row r="101" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A101" s="77" t="s">
-        <v>75</v>
-      </c>
-      <c r="B101" s="77"/>
-      <c r="C101" s="77"/>
-      <c r="D101" s="77"/>
-      <c r="E101" s="77"/>
+      <c r="B101" s="57"/>
+      <c r="C101" s="57"/>
+      <c r="D101" s="57"/>
+      <c r="E101" s="57"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="B10:J11"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B49:J49"/>
+    <mergeCell ref="B75:J75"/>
+    <mergeCell ref="B24:J25"/>
+    <mergeCell ref="B37:J38"/>
     <mergeCell ref="A98:H98"/>
     <mergeCell ref="A99:B99"/>
     <mergeCell ref="A100:B100"/>
@@ -4487,13 +4492,7 @@
     <mergeCell ref="B55:J56"/>
     <mergeCell ref="B69:J70"/>
     <mergeCell ref="B81:J82"/>
-    <mergeCell ref="B10:J11"/>
-    <mergeCell ref="B4:J4"/>
-    <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B49:J49"/>
-    <mergeCell ref="B75:J75"/>
-    <mergeCell ref="B24:J25"/>
-    <mergeCell ref="B37:J38"/>
+    <mergeCell ref="A96:B96"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="C96">
@@ -4554,7 +4553,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="76" t="s">
         <v>23</v>
       </c>
       <c r="B2" s="10">
@@ -4573,12 +4572,12 @@
       <c r="G2" s="5">
         <v>0</v>
       </c>
-      <c r="H2" s="64" t="s">
+      <c r="H2" s="76" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="65"/>
+      <c r="A3" s="77"/>
       <c r="B3" s="10">
         <v>1</v>
       </c>
@@ -4593,10 +4592,10 @@
       <c r="G3" s="5">
         <v>0</v>
       </c>
-      <c r="H3" s="65"/>
+      <c r="H3" s="77"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="65"/>
+      <c r="A4" s="77"/>
       <c r="B4" s="10">
         <v>1</v>
       </c>
@@ -4613,10 +4612,10 @@
       <c r="G4" s="5">
         <v>200</v>
       </c>
-      <c r="H4" s="65"/>
+      <c r="H4" s="77"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="65"/>
+      <c r="A5" s="77"/>
       <c r="B5" s="10">
         <v>1</v>
       </c>
@@ -4627,10 +4626,10 @@
       <c r="G5" s="5">
         <v>0</v>
       </c>
-      <c r="H5" s="65"/>
+      <c r="H5" s="77"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="65"/>
+      <c r="A6" s="77"/>
       <c r="B6" s="10">
         <v>1</v>
       </c>
@@ -4647,10 +4646,10 @@
       <c r="G6" s="5">
         <v>0</v>
       </c>
-      <c r="H6" s="65"/>
+      <c r="H6" s="77"/>
     </row>
     <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="65"/>
+      <c r="A7" s="77"/>
       <c r="B7" s="10">
         <v>1</v>
       </c>
@@ -4665,10 +4664,10 @@
       <c r="G7" s="5">
         <v>0</v>
       </c>
-      <c r="H7" s="65"/>
+      <c r="H7" s="77"/>
     </row>
     <row r="8" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="65"/>
+      <c r="A8" s="77"/>
       <c r="B8" s="24">
         <v>1</v>
       </c>
@@ -4685,10 +4684,10 @@
       <c r="G8" s="5">
         <v>50</v>
       </c>
-      <c r="H8" s="65"/>
+      <c r="H8" s="77"/>
     </row>
     <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="65"/>
+      <c r="A9" s="77"/>
       <c r="B9" s="24">
         <v>1</v>
       </c>
@@ -4698,10 +4697,10 @@
       <c r="D9" s="10"/>
       <c r="F9" s="1"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="65"/>
+      <c r="H9" s="77"/>
     </row>
     <row r="10" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="65"/>
+      <c r="A10" s="77"/>
       <c r="B10" s="24">
         <v>1</v>
       </c>
@@ -4714,10 +4713,10 @@
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="65"/>
+      <c r="H10" s="77"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="65"/>
+      <c r="A11" s="77"/>
       <c r="B11" s="10">
         <v>1</v>
       </c>
@@ -4728,10 +4727,10 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="65"/>
+      <c r="H11" s="77"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="65"/>
+      <c r="A12" s="77"/>
       <c r="B12" s="10">
         <v>1</v>
       </c>
@@ -4742,10 +4741,10 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="65"/>
+      <c r="H12" s="77"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="65"/>
+      <c r="A13" s="77"/>
       <c r="B13" s="10">
         <v>1</v>
       </c>
@@ -4756,10 +4755,10 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="65"/>
+      <c r="H13" s="77"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="65"/>
+      <c r="A14" s="77"/>
       <c r="B14" s="10">
         <v>1</v>
       </c>
@@ -4768,10 +4767,10 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="65"/>
+      <c r="H14" s="77"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="65"/>
+      <c r="A15" s="77"/>
       <c r="B15" s="10">
         <v>1</v>
       </c>
@@ -4782,10 +4781,10 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="5"/>
-      <c r="H15" s="65"/>
+      <c r="H15" s="77"/>
     </row>
     <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="65"/>
+      <c r="A16" s="77"/>
       <c r="B16" s="10">
         <v>1</v>
       </c>
@@ -4796,10 +4795,10 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="65"/>
+      <c r="H16" s="77"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="65"/>
+      <c r="A17" s="77"/>
       <c r="B17" s="24">
         <v>7</v>
       </c>
@@ -4808,70 +4807,70 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="65"/>
+      <c r="H17" s="77"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="65"/>
+      <c r="A18" s="77"/>
       <c r="B18" s="24"/>
       <c r="C18" s="35"/>
       <c r="D18" s="10"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="65"/>
+      <c r="H18" s="77"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="65"/>
+      <c r="A19" s="77"/>
       <c r="B19" s="24"/>
       <c r="C19" s="35"/>
       <c r="D19" s="10"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="65"/>
+      <c r="H19" s="77"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="65"/>
+      <c r="A20" s="77"/>
       <c r="B20" s="24"/>
       <c r="C20" s="35"/>
       <c r="D20" s="10"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="65"/>
+      <c r="H20" s="77"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="65"/>
+      <c r="A21" s="77"/>
       <c r="B21" s="24"/>
       <c r="C21" s="35"/>
       <c r="D21" s="10"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="65"/>
+      <c r="H21" s="77"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="65"/>
+      <c r="A22" s="77"/>
       <c r="B22" s="24"/>
       <c r="C22" s="35"/>
       <c r="D22" s="10"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="65"/>
+      <c r="H22" s="77"/>
     </row>
     <row r="23" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="65"/>
+      <c r="A23" s="77"/>
       <c r="B23" s="24"/>
       <c r="C23" s="36"/>
       <c r="D23" s="10"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="65"/>
+      <c r="H23" s="77"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="65"/>
+      <c r="A24" s="77"/>
       <c r="B24" s="10">
         <v>1</v>
       </c>
@@ -4882,10 +4881,10 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="65"/>
+      <c r="H24" s="77"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="65"/>
+      <c r="A25" s="77"/>
       <c r="B25" s="10">
         <v>1</v>
       </c>
@@ -4896,10 +4895,10 @@
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="65"/>
+      <c r="H25" s="77"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="65"/>
+      <c r="A26" s="77"/>
       <c r="B26" s="10">
         <v>1</v>
       </c>
@@ -4910,10 +4909,10 @@
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="65"/>
+      <c r="H26" s="77"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="65"/>
+      <c r="A27" s="77"/>
       <c r="B27" s="10">
         <v>1</v>
       </c>
@@ -4922,10 +4921,10 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="65"/>
+      <c r="H27" s="77"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="65"/>
+      <c r="A28" s="77"/>
       <c r="B28" s="10">
         <v>1</v>
       </c>
@@ -4934,10 +4933,10 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="65"/>
+      <c r="H28" s="77"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="65"/>
+      <c r="A29" s="77"/>
       <c r="B29" s="10">
         <v>1</v>
       </c>
@@ -4953,10 +4952,10 @@
       <c r="G29" s="5">
         <v>50</v>
       </c>
-      <c r="H29" s="65"/>
+      <c r="H29" s="77"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="65"/>
+      <c r="A30" s="77"/>
       <c r="B30" s="10">
         <v>6</v>
       </c>
@@ -4967,40 +4966,40 @@
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="65"/>
+      <c r="H30" s="77"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="65"/>
+      <c r="A31" s="77"/>
       <c r="B31" s="10"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="65"/>
+      <c r="H31" s="77"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="65"/>
+      <c r="A32" s="77"/>
       <c r="B32" s="10"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="5"/>
-      <c r="H32" s="65"/>
+      <c r="H32" s="77"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="65"/>
+      <c r="A33" s="77"/>
       <c r="B33" s="10"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="5"/>
-      <c r="H33" s="65"/>
+      <c r="H33" s="77"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="65"/>
+      <c r="A34" s="77"/>
       <c r="B34" s="10">
         <v>1</v>
       </c>
@@ -5013,10 +5012,10 @@
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="5"/>
-      <c r="H34" s="65"/>
+      <c r="H34" s="77"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="65"/>
+      <c r="A35" s="77"/>
       <c r="B35" s="10">
         <v>1</v>
       </c>
@@ -5027,10 +5026,10 @@
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
       <c r="G35" s="5"/>
-      <c r="H35" s="65"/>
+      <c r="H35" s="77"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="65"/>
+      <c r="A36" s="77"/>
       <c r="B36" s="10">
         <v>1</v>
       </c>
@@ -5047,10 +5046,10 @@
       <c r="G36" s="5">
         <v>200</v>
       </c>
-      <c r="H36" s="65"/>
+      <c r="H36" s="77"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="65"/>
+      <c r="A37" s="77"/>
       <c r="B37" s="10">
         <v>2</v>
       </c>
@@ -5061,10 +5060,10 @@
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="5"/>
-      <c r="H37" s="65"/>
+      <c r="H37" s="77"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="65"/>
+      <c r="A38" s="77"/>
       <c r="B38" s="10">
         <v>4</v>
       </c>
@@ -5079,10 +5078,10 @@
       <c r="G38" s="5">
         <v>250</v>
       </c>
-      <c r="H38" s="65"/>
+      <c r="H38" s="77"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="65"/>
+      <c r="A39" s="77"/>
       <c r="B39" s="10">
         <v>4</v>
       </c>
@@ -5097,37 +5096,37 @@
       <c r="G39" s="5">
         <v>250</v>
       </c>
-      <c r="H39" s="65"/>
+      <c r="H39" s="77"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="65"/>
+      <c r="A40" s="77"/>
       <c r="B40" s="10"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="5"/>
-      <c r="H40" s="65"/>
+      <c r="H40" s="77"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="65"/>
+      <c r="A41" s="77"/>
       <c r="B41" s="10"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="5"/>
-      <c r="H41" s="65"/>
+      <c r="H41" s="77"/>
     </row>
     <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="65"/>
+      <c r="A42" s="77"/>
       <c r="B42" s="12"/>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
       <c r="F42" s="13"/>
       <c r="G42" s="14"/>
-      <c r="H42" s="65"/>
+      <c r="H42" s="77"/>
     </row>
     <row r="43" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="15" t="s">
@@ -5354,21 +5353,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E4DE2CC379442A4D8483D9D7B1BA3E35" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3cbd871ac436bbcd94953c6f74650012">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1b380a0-b262-4a13-9203-497a21b8eee5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f82e0ce2898406bfa558450728792a3e" ns2:_="">
     <xsd:import namespace="a1b380a0-b262-4a13-9203-497a21b8eee5"/>
@@ -5506,24 +5490,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{456E5AF3-7BBF-4763-B83A-9DB8001DA7F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{160991D8-BA81-407D-9E91-473AD6B09576}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5F86897-A5B3-4CA1-BC45-17E92954BA24}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5539,4 +5521,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{160991D8-BA81-407D-9E91-473AD6B09576}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{456E5AF3-7BBF-4763-B83A-9DB8001DA7F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated excel for equipment
</commit_message>
<xml_diff>
--- a/calc_and_rack.xlsx
+++ b/calc_and_rack.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\l7aur\Desktop\CND\CNP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0318409-9D07-4107-AD2E-444995DA1C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB177BD1-40F2-4C22-B1EC-1930EFF56AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cable" sheetId="1" r:id="rId1"/>
     <sheet name="Fiber" sheetId="5" r:id="rId2"/>
-    <sheet name="MDF" sheetId="2" r:id="rId3"/>
-    <sheet name="IDF1" sheetId="3" r:id="rId4"/>
-    <sheet name="IDF..." sheetId="4" r:id="rId5"/>
+    <sheet name="Equipment" sheetId="6" r:id="rId3"/>
+    <sheet name="MDF" sheetId="2" r:id="rId4"/>
+    <sheet name="IDF1" sheetId="3" r:id="rId5"/>
+    <sheet name="IDF..." sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -109,7 +110,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="189">
   <si>
     <t>Room Nr</t>
   </si>
@@ -658,13 +659,31 @@
   </si>
   <si>
     <t>Target</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Choice 2</t>
+  </si>
+  <si>
+    <t>Equipment</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Choice 1 (CISCO)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -729,6 +748,13 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -827,7 +853,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="55">
+  <borders count="62">
     <border>
       <left/>
       <right/>
@@ -1529,11 +1555,96 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1595,6 +1706,93 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="15" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1606,8 +1804,6 @@
     <xf numFmtId="49" fontId="2" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1629,95 +1825,42 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2076,17 +2219,17 @@
       <c r="A4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="94" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
-      <c r="I4" s="62"/>
-      <c r="J4" s="63"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="86"/>
+      <c r="E4" s="86"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="86"/>
+      <c r="H4" s="86"/>
+      <c r="I4" s="86"/>
+      <c r="J4" s="87"/>
     </row>
     <row r="5" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -2272,31 +2415,31 @@
       <c r="A10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="55" t="s">
+      <c r="B10" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="56"/>
-      <c r="J10" s="57"/>
+      <c r="C10" s="89"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="89"/>
+      <c r="F10" s="89"/>
+      <c r="G10" s="89"/>
+      <c r="H10" s="89"/>
+      <c r="I10" s="89"/>
+      <c r="J10" s="90"/>
     </row>
     <row r="11" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="58"/>
-      <c r="C11" s="59"/>
-      <c r="D11" s="59"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="60"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="92"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="92"/>
+      <c r="G11" s="92"/>
+      <c r="H11" s="92"/>
+      <c r="I11" s="92"/>
+      <c r="J11" s="93"/>
     </row>
     <row r="12" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -2694,31 +2837,31 @@
       <c r="A24" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="55" t="s">
+      <c r="B24" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="56"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="56"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="56"/>
-      <c r="J24" s="57"/>
+      <c r="C24" s="89"/>
+      <c r="D24" s="89"/>
+      <c r="E24" s="89"/>
+      <c r="F24" s="89"/>
+      <c r="G24" s="89"/>
+      <c r="H24" s="89"/>
+      <c r="I24" s="89"/>
+      <c r="J24" s="90"/>
     </row>
     <row r="25" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="58"/>
-      <c r="C25" s="59"/>
-      <c r="D25" s="59"/>
-      <c r="E25" s="59"/>
-      <c r="F25" s="59"/>
-      <c r="G25" s="59"/>
-      <c r="H25" s="59"/>
-      <c r="I25" s="59"/>
-      <c r="J25" s="60"/>
+      <c r="B25" s="91"/>
+      <c r="C25" s="92"/>
+      <c r="D25" s="92"/>
+      <c r="E25" s="92"/>
+      <c r="F25" s="92"/>
+      <c r="G25" s="92"/>
+      <c r="H25" s="92"/>
+      <c r="I25" s="92"/>
+      <c r="J25" s="93"/>
     </row>
     <row r="26" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
@@ -2904,17 +3047,17 @@
       <c r="A31" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="61" t="s">
+      <c r="B31" s="94" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="62"/>
-      <c r="D31" s="62"/>
-      <c r="E31" s="62"/>
-      <c r="F31" s="62"/>
-      <c r="G31" s="62"/>
-      <c r="H31" s="62"/>
-      <c r="I31" s="62"/>
-      <c r="J31" s="63"/>
+      <c r="C31" s="86"/>
+      <c r="D31" s="86"/>
+      <c r="E31" s="86"/>
+      <c r="F31" s="86"/>
+      <c r="G31" s="86"/>
+      <c r="H31" s="86"/>
+      <c r="I31" s="86"/>
+      <c r="J31" s="87"/>
     </row>
     <row r="32" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
@@ -3100,31 +3243,31 @@
       <c r="A37" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="64" t="s">
+      <c r="B37" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="C37" s="56"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="56"/>
-      <c r="H37" s="56"/>
-      <c r="I37" s="56"/>
-      <c r="J37" s="57"/>
+      <c r="C37" s="89"/>
+      <c r="D37" s="89"/>
+      <c r="E37" s="89"/>
+      <c r="F37" s="89"/>
+      <c r="G37" s="89"/>
+      <c r="H37" s="89"/>
+      <c r="I37" s="89"/>
+      <c r="J37" s="90"/>
     </row>
     <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B38" s="58"/>
-      <c r="C38" s="59"/>
-      <c r="D38" s="59"/>
-      <c r="E38" s="59"/>
-      <c r="F38" s="59"/>
-      <c r="G38" s="59"/>
-      <c r="H38" s="59"/>
-      <c r="I38" s="59"/>
-      <c r="J38" s="60"/>
+      <c r="B38" s="91"/>
+      <c r="C38" s="92"/>
+      <c r="D38" s="92"/>
+      <c r="E38" s="92"/>
+      <c r="F38" s="92"/>
+      <c r="G38" s="92"/>
+      <c r="H38" s="92"/>
+      <c r="I38" s="92"/>
+      <c r="J38" s="93"/>
     </row>
     <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
@@ -3450,17 +3593,17 @@
       <c r="A49" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B49" s="73" t="s">
+      <c r="B49" s="85" t="s">
         <v>68</v>
       </c>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="63"/>
+      <c r="C49" s="86"/>
+      <c r="D49" s="86"/>
+      <c r="E49" s="86"/>
+      <c r="F49" s="86"/>
+      <c r="G49" s="86"/>
+      <c r="H49" s="86"/>
+      <c r="I49" s="86"/>
+      <c r="J49" s="87"/>
     </row>
     <row r="50" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
@@ -3646,31 +3789,31 @@
       <c r="A55" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B55" s="55" t="s">
+      <c r="B55" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="C55" s="56"/>
-      <c r="D55" s="56"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="56"/>
-      <c r="G55" s="56"/>
-      <c r="H55" s="56"/>
-      <c r="I55" s="56"/>
-      <c r="J55" s="57"/>
+      <c r="C55" s="89"/>
+      <c r="D55" s="89"/>
+      <c r="E55" s="89"/>
+      <c r="F55" s="89"/>
+      <c r="G55" s="89"/>
+      <c r="H55" s="89"/>
+      <c r="I55" s="89"/>
+      <c r="J55" s="90"/>
     </row>
     <row r="56" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B56" s="58"/>
-      <c r="C56" s="59"/>
-      <c r="D56" s="59"/>
-      <c r="E56" s="59"/>
-      <c r="F56" s="59"/>
-      <c r="G56" s="59"/>
-      <c r="H56" s="59"/>
-      <c r="I56" s="59"/>
-      <c r="J56" s="60"/>
+      <c r="B56" s="91"/>
+      <c r="C56" s="92"/>
+      <c r="D56" s="92"/>
+      <c r="E56" s="92"/>
+      <c r="F56" s="92"/>
+      <c r="G56" s="92"/>
+      <c r="H56" s="92"/>
+      <c r="I56" s="92"/>
+      <c r="J56" s="93"/>
     </row>
     <row r="57" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
@@ -4068,31 +4211,31 @@
       <c r="A69" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B69" s="55" t="s">
+      <c r="B69" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="C69" s="56"/>
-      <c r="D69" s="56"/>
-      <c r="E69" s="56"/>
-      <c r="F69" s="56"/>
-      <c r="G69" s="56"/>
-      <c r="H69" s="56"/>
-      <c r="I69" s="56"/>
-      <c r="J69" s="57"/>
+      <c r="C69" s="89"/>
+      <c r="D69" s="89"/>
+      <c r="E69" s="89"/>
+      <c r="F69" s="89"/>
+      <c r="G69" s="89"/>
+      <c r="H69" s="89"/>
+      <c r="I69" s="89"/>
+      <c r="J69" s="90"/>
     </row>
     <row r="70" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B70" s="58"/>
-      <c r="C70" s="59"/>
-      <c r="D70" s="59"/>
-      <c r="E70" s="59"/>
-      <c r="F70" s="59"/>
-      <c r="G70" s="59"/>
-      <c r="H70" s="59"/>
-      <c r="I70" s="59"/>
-      <c r="J70" s="60"/>
+      <c r="B70" s="91"/>
+      <c r="C70" s="92"/>
+      <c r="D70" s="92"/>
+      <c r="E70" s="92"/>
+      <c r="F70" s="92"/>
+      <c r="G70" s="92"/>
+      <c r="H70" s="92"/>
+      <c r="I70" s="92"/>
+      <c r="J70" s="93"/>
     </row>
     <row r="71" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
@@ -4242,17 +4385,17 @@
       <c r="A75" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="B75" s="61" t="s">
+      <c r="B75" s="94" t="s">
         <v>88</v>
       </c>
-      <c r="C75" s="62"/>
-      <c r="D75" s="62"/>
-      <c r="E75" s="62"/>
-      <c r="F75" s="62"/>
-      <c r="G75" s="62"/>
-      <c r="H75" s="62"/>
-      <c r="I75" s="62"/>
-      <c r="J75" s="63"/>
+      <c r="C75" s="86"/>
+      <c r="D75" s="86"/>
+      <c r="E75" s="86"/>
+      <c r="F75" s="86"/>
+      <c r="G75" s="86"/>
+      <c r="H75" s="86"/>
+      <c r="I75" s="86"/>
+      <c r="J75" s="87"/>
     </row>
     <row r="76" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
@@ -4438,31 +4581,31 @@
       <c r="A81" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="B81" s="64" t="s">
+      <c r="B81" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="C81" s="56"/>
-      <c r="D81" s="56"/>
-      <c r="E81" s="56"/>
-      <c r="F81" s="56"/>
-      <c r="G81" s="56"/>
-      <c r="H81" s="56"/>
-      <c r="I81" s="56"/>
-      <c r="J81" s="57"/>
+      <c r="C81" s="89"/>
+      <c r="D81" s="89"/>
+      <c r="E81" s="89"/>
+      <c r="F81" s="89"/>
+      <c r="G81" s="89"/>
+      <c r="H81" s="89"/>
+      <c r="I81" s="89"/>
+      <c r="J81" s="90"/>
     </row>
     <row r="82" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="B82" s="58"/>
-      <c r="C82" s="59"/>
-      <c r="D82" s="59"/>
-      <c r="E82" s="59"/>
-      <c r="F82" s="59"/>
-      <c r="G82" s="59"/>
-      <c r="H82" s="59"/>
-      <c r="I82" s="59"/>
-      <c r="J82" s="60"/>
+      <c r="B82" s="91"/>
+      <c r="C82" s="92"/>
+      <c r="D82" s="92"/>
+      <c r="E82" s="92"/>
+      <c r="F82" s="92"/>
+      <c r="G82" s="92"/>
+      <c r="H82" s="92"/>
+      <c r="I82" s="92"/>
+      <c r="J82" s="93"/>
     </row>
     <row r="83" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
@@ -4757,10 +4900,10 @@
       <c r="J96" s="15"/>
     </row>
     <row r="97" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="71" t="s">
+      <c r="A97" s="102" t="s">
         <v>126</v>
       </c>
-      <c r="B97" s="72"/>
+      <c r="B97" s="103"/>
       <c r="C97" s="18">
         <f>I91/(F91*2)</f>
         <v>53.358826815642459</v>
@@ -4773,42 +4916,42 @@
       <c r="J98" s="15"/>
     </row>
     <row r="99" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="70" t="s">
+      <c r="A99" s="101" t="s">
         <v>127</v>
       </c>
-      <c r="B99" s="66"/>
-      <c r="C99" s="66"/>
-      <c r="D99" s="66"/>
-      <c r="E99" s="66"/>
-      <c r="F99" s="66"/>
-      <c r="G99" s="66"/>
-      <c r="H99" s="67"/>
+      <c r="B99" s="97"/>
+      <c r="C99" s="97"/>
+      <c r="D99" s="97"/>
+      <c r="E99" s="97"/>
+      <c r="F99" s="97"/>
+      <c r="G99" s="97"/>
+      <c r="H99" s="98"/>
       <c r="J99" s="15"/>
     </row>
     <row r="100" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="69" t="s">
+      <c r="A100" s="100" t="s">
         <v>128</v>
       </c>
-      <c r="B100" s="67"/>
+      <c r="B100" s="98"/>
       <c r="H100" s="17"/>
       <c r="J100" s="15"/>
     </row>
     <row r="101" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="68" t="s">
+      <c r="A101" s="99" t="s">
         <v>129</v>
       </c>
-      <c r="B101" s="67"/>
+      <c r="B101" s="98"/>
       <c r="H101" s="17"/>
       <c r="J101" s="15"/>
     </row>
     <row r="102" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="65" t="s">
+      <c r="A102" s="96" t="s">
         <v>130</v>
       </c>
-      <c r="B102" s="66"/>
-      <c r="C102" s="66"/>
-      <c r="D102" s="66"/>
-      <c r="E102" s="67"/>
+      <c r="B102" s="97"/>
+      <c r="C102" s="97"/>
+      <c r="D102" s="97"/>
+      <c r="E102" s="98"/>
       <c r="H102" s="17"/>
       <c r="J102" s="15"/>
     </row>
@@ -8410,13 +8553,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B49:J49"/>
-    <mergeCell ref="B55:J56"/>
-    <mergeCell ref="B4:J4"/>
-    <mergeCell ref="B10:J11"/>
-    <mergeCell ref="B24:J25"/>
-    <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B37:J38"/>
     <mergeCell ref="B69:J70"/>
     <mergeCell ref="B75:J75"/>
     <mergeCell ref="B81:J82"/>
@@ -8425,6 +8561,13 @@
     <mergeCell ref="A100:B100"/>
     <mergeCell ref="A99:H99"/>
     <mergeCell ref="A97:B97"/>
+    <mergeCell ref="B49:J49"/>
+    <mergeCell ref="B55:J56"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B10:J11"/>
+    <mergeCell ref="B24:J25"/>
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B37:J38"/>
   </mergeCells>
   <conditionalFormatting sqref="C97">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="between">
@@ -8447,228 +8590,229 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="78"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="98" t="s">
+      <c r="A2" s="77" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="99"/>
-      <c r="C2" s="100" t="s">
+      <c r="B2" s="78"/>
+      <c r="C2" s="83" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="101"/>
-      <c r="E2" s="102" t="s">
+      <c r="D2" s="84"/>
+      <c r="E2" s="71" t="s">
         <v>116</v>
       </c>
-      <c r="F2" s="103"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="78"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="57"/>
     </row>
     <row r="3" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="94" t="s">
+      <c r="A3" s="79" t="s">
         <v>117</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="94" t="s">
+      <c r="B3" s="80"/>
+      <c r="C3" s="79" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="96"/>
-      <c r="E3" s="97">
+      <c r="D3" s="74"/>
+      <c r="E3" s="73">
         <v>35</v>
       </c>
-      <c r="F3" s="96"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="78"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="57"/>
     </row>
     <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="82" t="s">
+      <c r="A4" s="66" t="s">
         <v>119</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="82" t="s">
+      <c r="B4" s="81"/>
+      <c r="C4" s="66" t="s">
         <v>120</v>
       </c>
-      <c r="D4" s="85"/>
-      <c r="E4" s="92">
+      <c r="D4" s="67"/>
+      <c r="E4" s="75">
         <v>85</v>
       </c>
-      <c r="F4" s="85"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="77"/>
-      <c r="I4" s="76"/>
-      <c r="J4" s="78"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="57"/>
     </row>
     <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="82" t="s">
+      <c r="A5" s="66" t="s">
         <v>121</v>
       </c>
-      <c r="B5" s="90"/>
-      <c r="C5" s="82" t="s">
+      <c r="B5" s="81"/>
+      <c r="C5" s="66" t="s">
         <v>122</v>
       </c>
-      <c r="D5" s="85"/>
-      <c r="E5" s="92">
+      <c r="D5" s="67"/>
+      <c r="E5" s="75">
         <v>35</v>
       </c>
-      <c r="F5" s="85"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="77"/>
-      <c r="I5" s="76"/>
-      <c r="J5" s="78"/>
+      <c r="F5" s="67"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="55"/>
+      <c r="J5" s="57"/>
     </row>
     <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="104" t="s">
+      <c r="A6" s="60" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="105"/>
-      <c r="C6" s="104" t="s">
+      <c r="B6" s="61"/>
+      <c r="C6" s="60" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="105"/>
-      <c r="E6" s="104">
+      <c r="D6" s="61"/>
+      <c r="E6" s="60">
         <v>85</v>
       </c>
-      <c r="F6" s="105"/>
-      <c r="G6" s="80"/>
-      <c r="H6" s="77"/>
-      <c r="I6" s="76"/>
-      <c r="J6" s="78"/>
+      <c r="F6" s="61"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="57"/>
     </row>
     <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="104" t="s">
+      <c r="A7" s="60" t="s">
         <v>120</v>
       </c>
-      <c r="B7" s="105"/>
-      <c r="C7" s="104" t="s">
+      <c r="B7" s="61"/>
+      <c r="C7" s="60" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="105"/>
-      <c r="E7" s="104">
+      <c r="D7" s="61"/>
+      <c r="E7" s="60">
         <v>5</v>
       </c>
-      <c r="F7" s="105"/>
-      <c r="G7" s="80"/>
-      <c r="H7" s="77"/>
-      <c r="I7" s="76"/>
-      <c r="J7" s="78"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="55"/>
+      <c r="J7" s="57"/>
     </row>
     <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="104" t="s">
+      <c r="A8" s="60" t="s">
         <v>122</v>
       </c>
-      <c r="B8" s="105"/>
-      <c r="C8" s="104" t="s">
+      <c r="B8" s="61"/>
+      <c r="C8" s="60" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="105"/>
-      <c r="E8" s="104">
+      <c r="D8" s="61"/>
+      <c r="E8" s="60">
         <v>5</v>
       </c>
-      <c r="F8" s="105"/>
-      <c r="G8" s="80"/>
-      <c r="H8" s="77"/>
-      <c r="I8" s="76"/>
-      <c r="J8" s="78"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="57"/>
     </row>
     <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="104" t="s">
+      <c r="A9" s="60" t="s">
         <v>117</v>
       </c>
-      <c r="B9" s="105"/>
-      <c r="C9" s="104" t="s">
+      <c r="B9" s="61"/>
+      <c r="C9" s="60" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="105"/>
-      <c r="E9" s="104">
+      <c r="D9" s="61"/>
+      <c r="E9" s="60">
         <v>5</v>
       </c>
-      <c r="F9" s="105"/>
-      <c r="G9" s="80"/>
-      <c r="H9" s="77"/>
-      <c r="I9" s="76"/>
-      <c r="J9" s="78"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="55"/>
+      <c r="J9" s="57"/>
     </row>
     <row r="10" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="B10" s="91"/>
-      <c r="C10" s="83" t="s">
+      <c r="B10" s="82"/>
+      <c r="C10" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="86"/>
-      <c r="E10" s="93">
+      <c r="D10" s="69"/>
+      <c r="E10" s="76">
         <v>5</v>
       </c>
-      <c r="F10" s="86"/>
-      <c r="G10" s="80"/>
-      <c r="H10" s="77"/>
-      <c r="I10" s="76"/>
-      <c r="J10" s="78"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="57"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="76"/>
-      <c r="B11" s="76"/>
-      <c r="C11" s="76"/>
-      <c r="D11" s="76"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="77"/>
-      <c r="I11" s="76"/>
-      <c r="J11" s="78"/>
+      <c r="A11" s="55"/>
+      <c r="B11" s="55"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="55"/>
+      <c r="J11" s="57"/>
     </row>
     <row r="12" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="79" t="s">
+      <c r="A12" s="70" t="s">
         <v>125</v>
       </c>
-      <c r="B12" s="79"/>
-      <c r="C12" s="79"/>
-      <c r="D12" s="79"/>
-      <c r="E12" s="81">
+      <c r="B12" s="70"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="62">
         <f>SUM(E3:F10)</f>
         <v>260</v>
       </c>
-      <c r="F12" s="81"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="77"/>
-      <c r="I12" s="76"/>
-      <c r="J12" s="78"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="56"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="57"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="76"/>
-      <c r="B13" s="76"/>
-      <c r="C13" s="76"/>
-      <c r="D13" s="76"/>
-      <c r="E13" s="76"/>
-      <c r="F13" s="76"/>
-      <c r="G13" s="76"/>
-      <c r="H13" s="77"/>
-      <c r="I13" s="76"/>
-      <c r="J13" s="78"/>
+      <c r="A13" s="55"/>
+      <c r="B13" s="55"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="56"/>
+      <c r="I13" s="55"/>
+      <c r="J13" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
@@ -8680,26 +8824,84 @@
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="A12:D12"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="E5:F5"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="E10:F10"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2A52946-D4CE-40B0-A487-FBC087A60333}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="5" width="8.88671875" style="116"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="106" t="s">
+        <v>185</v>
+      </c>
+      <c r="B1" s="107"/>
+      <c r="C1" s="107"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="106" t="s">
+        <v>183</v>
+      </c>
+      <c r="B2" s="110" t="s">
+        <v>188</v>
+      </c>
+      <c r="C2" s="111"/>
+      <c r="D2" s="110" t="s">
+        <v>184</v>
+      </c>
+      <c r="E2" s="112"/>
+    </row>
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="109"/>
+      <c r="B3" s="113" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3" s="114" t="s">
+        <v>187</v>
+      </c>
+      <c r="D3" s="113" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="115" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B4" s="117"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:A3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H1000"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -8741,7 +8943,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="104" t="s">
         <v>138</v>
       </c>
       <c r="B2" s="23">
@@ -8760,12 +8962,12 @@
       <c r="G2" s="25">
         <v>0</v>
       </c>
-      <c r="H2" s="74" t="s">
+      <c r="H2" s="104" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="75"/>
+      <c r="A3" s="105"/>
       <c r="B3" s="23">
         <v>1</v>
       </c>
@@ -8780,10 +8982,10 @@
       <c r="G3" s="25">
         <v>0</v>
       </c>
-      <c r="H3" s="75"/>
+      <c r="H3" s="105"/>
     </row>
     <row r="4" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="75"/>
+      <c r="A4" s="105"/>
       <c r="B4" s="23">
         <v>1</v>
       </c>
@@ -8800,10 +9002,10 @@
       <c r="G4" s="25">
         <v>200</v>
       </c>
-      <c r="H4" s="75"/>
+      <c r="H4" s="105"/>
     </row>
     <row r="5" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="75"/>
+      <c r="A5" s="105"/>
       <c r="B5" s="23">
         <v>1</v>
       </c>
@@ -8814,10 +9016,10 @@
       <c r="G5" s="25">
         <v>0</v>
       </c>
-      <c r="H5" s="75"/>
+      <c r="H5" s="105"/>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="75"/>
+      <c r="A6" s="105"/>
       <c r="B6" s="23">
         <v>1</v>
       </c>
@@ -8834,10 +9036,10 @@
       <c r="G6" s="25">
         <v>0</v>
       </c>
-      <c r="H6" s="75"/>
+      <c r="H6" s="105"/>
     </row>
     <row r="7" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="75"/>
+      <c r="A7" s="105"/>
       <c r="B7" s="23">
         <v>1</v>
       </c>
@@ -8852,10 +9054,10 @@
       <c r="G7" s="25">
         <v>0</v>
       </c>
-      <c r="H7" s="75"/>
+      <c r="H7" s="105"/>
     </row>
     <row r="8" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="75"/>
+      <c r="A8" s="105"/>
       <c r="B8" s="27">
         <v>1</v>
       </c>
@@ -8872,10 +9074,10 @@
       <c r="G8" s="25">
         <v>50</v>
       </c>
-      <c r="H8" s="75"/>
+      <c r="H8" s="105"/>
     </row>
     <row r="9" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="75"/>
+      <c r="A9" s="105"/>
       <c r="B9" s="27">
         <v>1</v>
       </c>
@@ -8885,10 +9087,10 @@
       <c r="D9" s="23"/>
       <c r="F9" s="24"/>
       <c r="G9" s="25"/>
-      <c r="H9" s="75"/>
+      <c r="H9" s="105"/>
     </row>
     <row r="10" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="75"/>
+      <c r="A10" s="105"/>
       <c r="B10" s="27">
         <v>1</v>
       </c>
@@ -8901,10 +9103,10 @@
       </c>
       <c r="F10" s="24"/>
       <c r="G10" s="25"/>
-      <c r="H10" s="75"/>
+      <c r="H10" s="105"/>
     </row>
     <row r="11" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="75"/>
+      <c r="A11" s="105"/>
       <c r="B11" s="23">
         <v>1</v>
       </c>
@@ -8915,10 +9117,10 @@
       <c r="E11" s="24"/>
       <c r="F11" s="24"/>
       <c r="G11" s="25"/>
-      <c r="H11" s="75"/>
+      <c r="H11" s="105"/>
     </row>
     <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="75"/>
+      <c r="A12" s="105"/>
       <c r="B12" s="23">
         <v>1</v>
       </c>
@@ -8929,10 +9131,10 @@
       <c r="E12" s="24"/>
       <c r="F12" s="24"/>
       <c r="G12" s="25"/>
-      <c r="H12" s="75"/>
+      <c r="H12" s="105"/>
     </row>
     <row r="13" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="75"/>
+      <c r="A13" s="105"/>
       <c r="B13" s="23">
         <v>1</v>
       </c>
@@ -8943,10 +9145,10 @@
       <c r="E13" s="24"/>
       <c r="F13" s="24"/>
       <c r="G13" s="25"/>
-      <c r="H13" s="75"/>
+      <c r="H13" s="105"/>
     </row>
     <row r="14" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="75"/>
+      <c r="A14" s="105"/>
       <c r="B14" s="23">
         <v>1</v>
       </c>
@@ -8955,10 +9157,10 @@
       <c r="E14" s="24"/>
       <c r="F14" s="24"/>
       <c r="G14" s="25"/>
-      <c r="H14" s="75"/>
+      <c r="H14" s="105"/>
     </row>
     <row r="15" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="75"/>
+      <c r="A15" s="105"/>
       <c r="B15" s="23">
         <v>1</v>
       </c>
@@ -8969,10 +9171,10 @@
       <c r="E15" s="24"/>
       <c r="F15" s="24"/>
       <c r="G15" s="25"/>
-      <c r="H15" s="75"/>
+      <c r="H15" s="105"/>
     </row>
     <row r="16" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="75"/>
+      <c r="A16" s="105"/>
       <c r="B16" s="23">
         <v>1</v>
       </c>
@@ -8983,10 +9185,10 @@
       <c r="E16" s="24"/>
       <c r="F16" s="24"/>
       <c r="G16" s="25"/>
-      <c r="H16" s="75"/>
+      <c r="H16" s="105"/>
     </row>
     <row r="17" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="75"/>
+      <c r="A17" s="105"/>
       <c r="B17" s="27">
         <v>7</v>
       </c>
@@ -8995,70 +9197,70 @@
       <c r="E17" s="24"/>
       <c r="F17" s="24"/>
       <c r="G17" s="25"/>
-      <c r="H17" s="75"/>
+      <c r="H17" s="105"/>
     </row>
     <row r="18" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="75"/>
+      <c r="A18" s="105"/>
       <c r="B18" s="27"/>
       <c r="C18" s="33"/>
       <c r="D18" s="23"/>
       <c r="E18" s="24"/>
       <c r="F18" s="24"/>
       <c r="G18" s="25"/>
-      <c r="H18" s="75"/>
+      <c r="H18" s="105"/>
     </row>
     <row r="19" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="75"/>
+      <c r="A19" s="105"/>
       <c r="B19" s="27"/>
       <c r="C19" s="33"/>
       <c r="D19" s="23"/>
       <c r="E19" s="24"/>
       <c r="F19" s="24"/>
       <c r="G19" s="25"/>
-      <c r="H19" s="75"/>
+      <c r="H19" s="105"/>
     </row>
     <row r="20" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="75"/>
+      <c r="A20" s="105"/>
       <c r="B20" s="27"/>
       <c r="C20" s="33"/>
       <c r="D20" s="23"/>
       <c r="E20" s="24"/>
       <c r="F20" s="24"/>
       <c r="G20" s="25"/>
-      <c r="H20" s="75"/>
+      <c r="H20" s="105"/>
     </row>
     <row r="21" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="75"/>
+      <c r="A21" s="105"/>
       <c r="B21" s="27"/>
       <c r="C21" s="33"/>
       <c r="D21" s="23"/>
       <c r="E21" s="24"/>
       <c r="F21" s="24"/>
       <c r="G21" s="25"/>
-      <c r="H21" s="75"/>
+      <c r="H21" s="105"/>
     </row>
     <row r="22" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="75"/>
+      <c r="A22" s="105"/>
       <c r="B22" s="27"/>
       <c r="C22" s="33"/>
       <c r="D22" s="23"/>
       <c r="E22" s="24"/>
       <c r="F22" s="24"/>
       <c r="G22" s="25"/>
-      <c r="H22" s="75"/>
+      <c r="H22" s="105"/>
     </row>
     <row r="23" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="75"/>
+      <c r="A23" s="105"/>
       <c r="B23" s="27"/>
       <c r="C23" s="34"/>
       <c r="D23" s="23"/>
       <c r="E23" s="24"/>
       <c r="F23" s="24"/>
       <c r="G23" s="25"/>
-      <c r="H23" s="75"/>
+      <c r="H23" s="105"/>
     </row>
     <row r="24" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="75"/>
+      <c r="A24" s="105"/>
       <c r="B24" s="23">
         <v>1</v>
       </c>
@@ -9069,10 +9271,10 @@
       <c r="E24" s="24"/>
       <c r="F24" s="24"/>
       <c r="G24" s="25"/>
-      <c r="H24" s="75"/>
+      <c r="H24" s="105"/>
     </row>
     <row r="25" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="75"/>
+      <c r="A25" s="105"/>
       <c r="B25" s="23">
         <v>1</v>
       </c>
@@ -9083,10 +9285,10 @@
       <c r="E25" s="24"/>
       <c r="F25" s="24"/>
       <c r="G25" s="25"/>
-      <c r="H25" s="75"/>
+      <c r="H25" s="105"/>
     </row>
     <row r="26" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="75"/>
+      <c r="A26" s="105"/>
       <c r="B26" s="23">
         <v>1</v>
       </c>
@@ -9097,10 +9299,10 @@
       <c r="E26" s="24"/>
       <c r="F26" s="24"/>
       <c r="G26" s="25"/>
-      <c r="H26" s="75"/>
+      <c r="H26" s="105"/>
     </row>
     <row r="27" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="75"/>
+      <c r="A27" s="105"/>
       <c r="B27" s="23">
         <v>1</v>
       </c>
@@ -9109,10 +9311,10 @@
       <c r="E27" s="24"/>
       <c r="F27" s="24"/>
       <c r="G27" s="25"/>
-      <c r="H27" s="75"/>
+      <c r="H27" s="105"/>
     </row>
     <row r="28" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="75"/>
+      <c r="A28" s="105"/>
       <c r="B28" s="23">
         <v>1</v>
       </c>
@@ -9121,10 +9323,10 @@
       <c r="E28" s="24"/>
       <c r="F28" s="24"/>
       <c r="G28" s="25"/>
-      <c r="H28" s="75"/>
+      <c r="H28" s="105"/>
     </row>
     <row r="29" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="75"/>
+      <c r="A29" s="105"/>
       <c r="B29" s="23">
         <v>1</v>
       </c>
@@ -9140,10 +9342,10 @@
       <c r="G29" s="25">
         <v>50</v>
       </c>
-      <c r="H29" s="75"/>
+      <c r="H29" s="105"/>
     </row>
     <row r="30" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="75"/>
+      <c r="A30" s="105"/>
       <c r="B30" s="23">
         <v>6</v>
       </c>
@@ -9154,40 +9356,40 @@
       <c r="E30" s="24"/>
       <c r="F30" s="24"/>
       <c r="G30" s="25"/>
-      <c r="H30" s="75"/>
+      <c r="H30" s="105"/>
     </row>
     <row r="31" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="75"/>
+      <c r="A31" s="105"/>
       <c r="B31" s="23"/>
       <c r="C31" s="24"/>
       <c r="D31" s="24"/>
       <c r="E31" s="24"/>
       <c r="F31" s="24"/>
       <c r="G31" s="25"/>
-      <c r="H31" s="75"/>
+      <c r="H31" s="105"/>
     </row>
     <row r="32" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="75"/>
+      <c r="A32" s="105"/>
       <c r="B32" s="23"/>
       <c r="C32" s="24"/>
       <c r="D32" s="24"/>
       <c r="E32" s="24"/>
       <c r="F32" s="24"/>
       <c r="G32" s="25"/>
-      <c r="H32" s="75"/>
+      <c r="H32" s="105"/>
     </row>
     <row r="33" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="75"/>
+      <c r="A33" s="105"/>
       <c r="B33" s="23"/>
       <c r="C33" s="24"/>
       <c r="D33" s="24"/>
       <c r="E33" s="24"/>
       <c r="F33" s="24"/>
       <c r="G33" s="25"/>
-      <c r="H33" s="75"/>
+      <c r="H33" s="105"/>
     </row>
     <row r="34" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="75"/>
+      <c r="A34" s="105"/>
       <c r="B34" s="23">
         <v>1</v>
       </c>
@@ -9200,10 +9402,10 @@
       </c>
       <c r="F34" s="24"/>
       <c r="G34" s="25"/>
-      <c r="H34" s="75"/>
+      <c r="H34" s="105"/>
     </row>
     <row r="35" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="75"/>
+      <c r="A35" s="105"/>
       <c r="B35" s="23">
         <v>1</v>
       </c>
@@ -9214,10 +9416,10 @@
       <c r="E35" s="24"/>
       <c r="F35" s="24"/>
       <c r="G35" s="25"/>
-      <c r="H35" s="75"/>
+      <c r="H35" s="105"/>
     </row>
     <row r="36" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="75"/>
+      <c r="A36" s="105"/>
       <c r="B36" s="23">
         <v>1</v>
       </c>
@@ -9234,10 +9436,10 @@
       <c r="G36" s="25">
         <v>200</v>
       </c>
-      <c r="H36" s="75"/>
+      <c r="H36" s="105"/>
     </row>
     <row r="37" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="75"/>
+      <c r="A37" s="105"/>
       <c r="B37" s="23">
         <v>2</v>
       </c>
@@ -9248,10 +9450,10 @@
       <c r="E37" s="24"/>
       <c r="F37" s="24"/>
       <c r="G37" s="25"/>
-      <c r="H37" s="75"/>
+      <c r="H37" s="105"/>
     </row>
     <row r="38" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="75"/>
+      <c r="A38" s="105"/>
       <c r="B38" s="23">
         <v>4</v>
       </c>
@@ -9266,10 +9468,10 @@
       <c r="G38" s="25">
         <v>250</v>
       </c>
-      <c r="H38" s="75"/>
+      <c r="H38" s="105"/>
     </row>
     <row r="39" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="75"/>
+      <c r="A39" s="105"/>
       <c r="B39" s="23">
         <v>4</v>
       </c>
@@ -9284,37 +9486,37 @@
       <c r="G39" s="25">
         <v>250</v>
       </c>
-      <c r="H39" s="75"/>
+      <c r="H39" s="105"/>
     </row>
     <row r="40" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="75"/>
+      <c r="A40" s="105"/>
       <c r="B40" s="23"/>
       <c r="C40" s="24"/>
       <c r="D40" s="24"/>
       <c r="E40" s="24"/>
       <c r="F40" s="24"/>
       <c r="G40" s="25"/>
-      <c r="H40" s="75"/>
+      <c r="H40" s="105"/>
     </row>
     <row r="41" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="75"/>
+      <c r="A41" s="105"/>
       <c r="B41" s="23"/>
       <c r="C41" s="24"/>
       <c r="D41" s="24"/>
       <c r="E41" s="24"/>
       <c r="F41" s="24"/>
       <c r="G41" s="25"/>
-      <c r="H41" s="75"/>
+      <c r="H41" s="105"/>
     </row>
     <row r="42" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="75"/>
+      <c r="A42" s="105"/>
       <c r="B42" s="36"/>
       <c r="C42" s="26"/>
       <c r="D42" s="26"/>
       <c r="E42" s="26"/>
       <c r="F42" s="26"/>
       <c r="G42" s="37"/>
-      <c r="H42" s="75"/>
+      <c r="H42" s="105"/>
     </row>
     <row r="43" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="38" t="s">
@@ -10458,7 +10660,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A1000"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -11472,7 +11674,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A1000"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>